<commit_message>
fix(project-management): compute PERT figures with a bundled summarizer and harden the SOW pipeline
- summarize.py computes the workbook figures from excel-input.json,
  validates the input and checks the generated formulas (optional
  LibreOffice recalc); Phase 6 and the SOW backfill use it
- full input schema documented; examples cleaned and anonymized;
  8/80 in person-days per activity
- agents return drafts and questions, the skill runs the checkpoints;
  sow-estimate handoff read by PERT Phase 1
- high risk is PxI >= 10 everywhere; openpyxl checked before use
- one configuration section, per-estimate working folders, versioned
  outputs that never overwrite
- DOCX via optional document converter; sow-review half-open grades and
  report language; narrower sow-write triggers
</commit_message>
<xml_diff>
--- a/project-management/skills/pmo-pert-estimate/examples/scenario-1-website-redesign/pert-estimate.xlsx
+++ b/project-management/skills/pmo-pert-estimate/examples/scenario-1-website-redesign/pert-estimate.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +46,10 @@
     <font>
       <b val="1"/>
       <color rgb="FF9C0006"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
     </font>
   </fonts>
   <fills count="7">
@@ -96,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,6 +147,7 @@
     <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -2546,117 +2551,117 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Client delays sign-off on mockups, blocking development start</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
         <is>
           <t>Organisational</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="20" t="inlineStr">
         <is>
           <t>1, 2</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="20">
         <f>E2*F2</f>
         <v/>
       </c>
-      <c r="H2">
+      <c r="H2" s="20">
         <f>IF(G2&gt;=15,"CRITICAL",IF(G2&gt;=10,"HIGH",IF(G2&gt;=5,"MEDIUM","LOW")))</f>
         <v/>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="20" t="inlineStr">
         <is>
           <t>Mitigate</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="20" t="inlineStr">
         <is>
           <t>Define clear sign-off deadlines in contract; escalate after 3 business days</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="20" t="inlineStr">
         <is>
           <t>DSG</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="20">
         <f>L2*450</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Content migration takes longer due to inconsistent legacy data formats</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>Technical</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="20">
         <f>E3*F3</f>
         <v/>
       </c>
-      <c r="H3">
+      <c r="H3" s="20">
         <f>IF(G3&gt;=15,"CRITICAL",IF(G3&gt;=10,"HIGH",IF(G3&gt;=5,"MEDIUM","LOW")))</f>
         <v/>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>Mitigate</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="20" t="inlineStr">
         <is>
           <t>Audit legacy content before migration; prepare transformation scripts</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="20" t="inlineStr">
         <is>
           <t>DEV</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="20">
         <f>L3*450</f>
         <v/>
       </c>
@@ -3145,12 +3150,12 @@
           <t>Calendar Duration (weeks)</t>
         </is>
       </c>
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="21" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>Effort by Team (PD)</t>
         </is>
@@ -3167,7 +3172,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>Sensitivity Scenarios</t>
         </is>

</xml_diff>